<commit_message>
Update PE Programação e Controle de Sistemas Robóticos FRC.xlsx
</commit_message>
<xml_diff>
--- a/Programação e Controle de Sistemas Robóticos FRC/PE Programação e Controle de Sistemas Robóticos FRC.xlsx
+++ b/Programação e Controle de Sistemas Robóticos FRC/PE Programação e Controle de Sistemas Robóticos FRC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djair.oliveira\Documents\GitHub\Curso 2026\Programação e Controle de Sistemas Robóticos FRC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFD3A0D-72DD-437A-85E6-9B85C97A3FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C31AB91D-83D8-4E56-A173-DD6188C6D890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="76">
   <si>
     <t xml:space="preserve">                      </t>
   </si>
@@ -553,9 +553,6 @@
     <t xml:space="preserve">Unidade Operacional:       </t>
   </si>
   <si>
-    <t>Condutores de processos robotizados</t>
-  </si>
-  <si>
     <t>Qualificação Profissional</t>
   </si>
   <si>
@@ -600,9 +597,6 @@
   </si>
   <si>
     <t>20 Horas</t>
-  </si>
-  <si>
-    <t>Programação e Controle de Sistemas Robóticos FRC</t>
   </si>
   <si>
     <t>160 Horas</t>
@@ -684,6 +678,9 @@
   </si>
   <si>
     <t xml:space="preserve">40 Horas </t>
+  </si>
+  <si>
+    <t>Desenvolvimento e Programação de Sistemas Robóticos</t>
   </si>
 </sst>
 </file>
@@ -992,7 +989,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1065,11 +1062,97 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1079,94 +1162,6 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1178,6 +1173,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1690,7 +1691,7 @@
   <sheetData>
     <row r="1" spans="2:8" ht="10.5" customHeight="1"/>
     <row r="2" spans="2:8" ht="33" customHeight="1">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="36" t="s">
@@ -1705,7 +1706,7 @@
       <c r="H2" s="31"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1">
-      <c r="B3" s="28"/>
+      <c r="B3" s="27"/>
       <c r="C3" s="39"/>
       <c r="D3" s="40"/>
       <c r="E3" s="41"/>
@@ -1720,7 +1721,7 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B4" s="29"/>
+      <c r="B4" s="28"/>
       <c r="C4" s="42"/>
       <c r="D4" s="43"/>
       <c r="E4" s="44"/>
@@ -1732,29 +1733,29 @@
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="51"/>
-    </row>
-    <row r="7" spans="2:8" ht="15.6">
+      <c r="C6" s="48"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
+    </row>
+    <row r="7" spans="2:8" ht="30">
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="48" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
     </row>
     <row r="8" spans="2:8" ht="15.6">
       <c r="B8" s="2" t="s">
@@ -1764,12 +1765,12 @@
       <c r="D8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="48" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="48"/>
+      <c r="E8" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="2:8" ht="15.6">
       <c r="B9" s="2" t="s">
@@ -1779,53 +1780,53 @@
       <c r="D9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
-    </row>
-    <row r="10" spans="2:8" ht="15.6">
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+    </row>
+    <row r="10" spans="2:8" ht="30">
       <c r="B10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>58</v>
+      <c r="C10" s="23" t="s">
+        <v>75</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
+      <c r="E10" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="2:8" ht="78.75" customHeight="1">
       <c r="B11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="48" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="48"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="48"/>
-      <c r="G11" s="48"/>
-      <c r="H11" s="48"/>
+      <c r="C11" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="2:8" ht="73.5" customHeight="1">
       <c r="B12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="48"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="48"/>
-      <c r="G12" s="48"/>
-      <c r="H12" s="48"/>
+      <c r="C12" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="2:8" s="1" customFormat="1" ht="15.6">
       <c r="B13" s="7"/>
@@ -1846,175 +1847,175 @@
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1">
-      <c r="B15" s="52" t="s">
+      <c r="B15" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52" t="s">
+      <c r="D15" s="24"/>
+      <c r="E15" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="52" t="s">
+      <c r="F15" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="52" t="s">
+      <c r="G15" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="24" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="36" customHeight="1">
-      <c r="B16" s="52"/>
+      <c r="B16" s="24"/>
       <c r="C16" s="8" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="2:8" ht="93" customHeight="1">
       <c r="B17" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="150">
       <c r="B18" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H18" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="210">
       <c r="B19" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F19" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19" s="20" t="s">
         <v>52</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H19" s="20" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="270">
       <c r="B20" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E20" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="H20" s="20" t="s">
         <v>54</v>
-      </c>
-      <c r="F20" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H20" s="20" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="270">
       <c r="B21" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="E21" s="20" t="s">
+      <c r="H21" s="20" t="s">
         <v>54</v>
-      </c>
-      <c r="F21" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H21" s="20" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="210">
       <c r="B22" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F22" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="H22" s="20" t="s">
         <v>52</v>
-      </c>
-      <c r="G22" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H22" s="20" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="15">
@@ -2175,21 +2176,21 @@
       <c r="B39" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="53"/>
+      <c r="H39" s="53"/>
     </row>
     <row r="40" spans="2:8" ht="15.6">
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
     </row>
     <row r="41" spans="2:8" ht="15.6">
       <c r="B41" s="9" t="s">
@@ -2219,21 +2220,21 @@
       <c r="B43" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
+      <c r="C43" s="53"/>
+      <c r="D43" s="53"/>
+      <c r="E43" s="53"/>
+      <c r="F43" s="53"/>
+      <c r="G43" s="53"/>
+      <c r="H43" s="53"/>
     </row>
     <row r="44" spans="2:8" ht="15.6">
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="29"/>
     </row>
     <row r="45" spans="2:8" ht="15.6">
       <c r="B45" s="9" t="s">
@@ -2263,21 +2264,21 @@
       <c r="B47" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
+      <c r="C47" s="53"/>
+      <c r="D47" s="53"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="53"/>
+      <c r="G47" s="53"/>
+      <c r="H47" s="53"/>
     </row>
     <row r="48" spans="2:8" ht="15.6">
-      <c r="B48" s="30"/>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
     </row>
     <row r="49" spans="2:8" ht="15.6">
       <c r="B49" s="9" t="s">
@@ -2298,21 +2299,21 @@
       <c r="B50" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
-      <c r="H50" s="26"/>
+      <c r="C50" s="53"/>
+      <c r="D50" s="53"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="53"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="53"/>
     </row>
     <row r="51" spans="2:8" ht="15.6">
-      <c r="B51" s="24"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-      <c r="G51" s="24"/>
-      <c r="H51" s="24"/>
+      <c r="B51" s="30"/>
+      <c r="C51" s="30"/>
+      <c r="D51" s="30"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
     </row>
     <row r="52" spans="2:8" ht="15.6">
       <c r="B52" s="9" t="s">
@@ -2333,21 +2334,21 @@
       <c r="B53" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
-      <c r="H53" s="26"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="53"/>
+      <c r="H53" s="53"/>
     </row>
     <row r="54" spans="2:8" ht="15.6">
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="23"/>
-      <c r="F54" s="23"/>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
+      <c r="B54" s="51"/>
+      <c r="C54" s="51"/>
+      <c r="D54" s="51"/>
+      <c r="E54" s="51"/>
+      <c r="F54" s="51"/>
+      <c r="G54" s="51"/>
+      <c r="H54" s="51"/>
     </row>
     <row r="55" spans="2:8" ht="15.6">
       <c r="B55" s="9" t="s">
@@ -2368,21 +2369,21 @@
       <c r="B56" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
-      <c r="G56" s="26"/>
-      <c r="H56" s="26"/>
+      <c r="C56" s="53"/>
+      <c r="D56" s="53"/>
+      <c r="E56" s="53"/>
+      <c r="F56" s="53"/>
+      <c r="G56" s="53"/>
+      <c r="H56" s="53"/>
     </row>
     <row r="57" spans="2:8" ht="15.6">
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="24"/>
-      <c r="E57" s="24"/>
-      <c r="F57" s="24"/>
-      <c r="G57" s="24"/>
-      <c r="H57" s="24"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+      <c r="D57" s="30"/>
+      <c r="E57" s="30"/>
+      <c r="F57" s="30"/>
+      <c r="G57" s="30"/>
+      <c r="H57" s="30"/>
     </row>
     <row r="58" spans="2:8" ht="15.6">
       <c r="B58" s="9" t="s">
@@ -2412,21 +2413,21 @@
       <c r="B60" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="26"/>
+      <c r="C60" s="53"/>
+      <c r="D60" s="53"/>
+      <c r="E60" s="53"/>
+      <c r="F60" s="53"/>
+      <c r="G60" s="53"/>
+      <c r="H60" s="53"/>
     </row>
     <row r="61" spans="2:8" ht="15.6">
-      <c r="B61" s="24"/>
-      <c r="C61" s="24"/>
-      <c r="D61" s="24"/>
-      <c r="E61" s="24"/>
-      <c r="F61" s="24"/>
-      <c r="G61" s="24"/>
-      <c r="H61" s="24"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="30"/>
+      <c r="E61" s="30"/>
+      <c r="F61" s="30"/>
+      <c r="G61" s="30"/>
+      <c r="H61" s="30"/>
     </row>
     <row r="62" spans="2:8" ht="23.25" customHeight="1">
       <c r="B62" s="9"/>
@@ -2501,10 +2502,10 @@
         <v>41</v>
       </c>
       <c r="D69" s="16"/>
-      <c r="E69" s="25" t="s">
+      <c r="E69" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="F69" s="25"/>
+      <c r="F69" s="52"/>
       <c r="G69" s="16"/>
       <c r="H69" s="11"/>
     </row>
@@ -2529,14 +2530,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ccZpZMWR273qlvLUtwEZJUOxiJ5jmkvTa0dLE26tSkBqPY5m3mRoMHNqIjYbEpq7rzB081kTHOTXRSPleNsf/g==" saltValue="jJlEsT6/mtXyWYTyFwVD1Q==" spinCount="100000" sheet="1" formatColumns="0" formatRows="0" insertRows="0"/>
   <mergeCells count="35">
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B57:H57"/>
+    <mergeCell ref="B61:H61"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C53:H53"/>
+    <mergeCell ref="C56:H56"/>
+    <mergeCell ref="C60:H60"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B40:H40"/>
     <mergeCell ref="B44:H44"/>
@@ -2553,17 +2557,14 @@
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="H15:H16"/>
-    <mergeCell ref="B54:H54"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="B61:H61"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="C53:H53"/>
-    <mergeCell ref="C56:H56"/>
-    <mergeCell ref="C60:H60"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="C11:H11"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2594,14 +2595,14 @@
   <sheetData>
     <row r="1" spans="2:8" ht="10.5" customHeight="1"/>
     <row r="2" spans="2:8" ht="33" customHeight="1">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="58" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="57" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
       <c r="F2" s="31" t="s">
         <v>2</v>
       </c>
@@ -2609,10 +2610,10 @@
       <c r="H2" s="31"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1">
-      <c r="B3" s="54"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
       <c r="F3" s="32" t="s">
         <v>3</v>
       </c>
@@ -2624,10 +2625,10 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B4" s="54"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
       <c r="F4" s="32"/>
       <c r="G4" s="35"/>
       <c r="H4" s="35"/>
@@ -2636,12 +2637,12 @@
       <c r="B6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="55"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="57"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="56"/>
     </row>
     <row r="7" spans="2:8" ht="15.6">
       <c r="B7" s="2" t="s">
@@ -2651,10 +2652,10 @@
       <c r="D7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
     </row>
     <row r="8" spans="2:8" ht="15.6">
       <c r="B8" s="2" t="s">
@@ -2664,10 +2665,10 @@
       <c r="D8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="48"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="2:8" ht="15.6">
       <c r="B9" s="2" t="s">
@@ -2677,10 +2678,10 @@
       <c r="D9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" spans="2:8" ht="15.6">
       <c r="B10" s="2" t="s">
@@ -2690,32 +2691,32 @@
       <c r="D10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="2:8" ht="78.75" customHeight="1">
       <c r="B11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="48"/>
-      <c r="G11" s="48"/>
-      <c r="H11" s="48"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="2:8" ht="73.5" customHeight="1" thickBot="1">
       <c r="B12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="48"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="48"/>
-      <c r="G12" s="48"/>
-      <c r="H12" s="48"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="2:8" s="1" customFormat="1" ht="15.6">
       <c r="B13" s="7"/>
@@ -2736,38 +2737,38 @@
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1">
-      <c r="B15" s="52" t="s">
+      <c r="B15" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52" t="s">
+      <c r="D15" s="24"/>
+      <c r="E15" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="52" t="s">
+      <c r="F15" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="52" t="s">
+      <c r="G15" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="24" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="36" customHeight="1">
-      <c r="B16" s="52"/>
+      <c r="B16" s="24"/>
       <c r="C16" s="8" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="2:8" ht="15">
       <c r="B17" s="3"/>
@@ -2981,12 +2982,12 @@
       <c r="B39" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="53"/>
+      <c r="H39" s="53"/>
     </row>
     <row r="40" spans="2:8" ht="15.6">
       <c r="B40" s="9"/>
@@ -3025,12 +3026,12 @@
       <c r="B43" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
+      <c r="C43" s="53"/>
+      <c r="D43" s="53"/>
+      <c r="E43" s="53"/>
+      <c r="F43" s="53"/>
+      <c r="G43" s="53"/>
+      <c r="H43" s="53"/>
     </row>
     <row r="44" spans="2:8" ht="15.6">
       <c r="B44" s="9"/>
@@ -3069,12 +3070,12 @@
       <c r="B47" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
+      <c r="C47" s="53"/>
+      <c r="D47" s="53"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="53"/>
+      <c r="G47" s="53"/>
+      <c r="H47" s="53"/>
     </row>
     <row r="48" spans="2:8" ht="15.6">
       <c r="B48" s="9"/>
@@ -3104,12 +3105,12 @@
       <c r="B50" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
-      <c r="H50" s="26"/>
+      <c r="C50" s="53"/>
+      <c r="D50" s="53"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="53"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="53"/>
     </row>
     <row r="51" spans="2:8" ht="15.6">
       <c r="B51" s="9"/>
@@ -3139,12 +3140,12 @@
       <c r="B53" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
-      <c r="H53" s="26"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="53"/>
+      <c r="H53" s="53"/>
     </row>
     <row r="54" spans="2:8" ht="15.6">
       <c r="B54" s="7"/>
@@ -3174,12 +3175,12 @@
       <c r="B56" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
-      <c r="G56" s="26"/>
-      <c r="H56" s="26"/>
+      <c r="C56" s="53"/>
+      <c r="D56" s="53"/>
+      <c r="E56" s="53"/>
+      <c r="F56" s="53"/>
+      <c r="G56" s="53"/>
+      <c r="H56" s="53"/>
     </row>
     <row r="57" spans="2:8" ht="15.6">
       <c r="B57" s="9"/>
@@ -3218,12 +3219,12 @@
       <c r="B60" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="26"/>
+      <c r="C60" s="53"/>
+      <c r="D60" s="53"/>
+      <c r="E60" s="53"/>
+      <c r="F60" s="53"/>
+      <c r="G60" s="53"/>
+      <c r="H60" s="53"/>
     </row>
     <row r="61" spans="2:8" ht="15.6">
       <c r="B61" s="9"/>
@@ -3298,10 +3299,10 @@
         <v>41</v>
       </c>
       <c r="D68" s="16"/>
-      <c r="E68" s="25" t="s">
+      <c r="E68" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="F68" s="25"/>
+      <c r="F68" s="52"/>
       <c r="G68" s="16"/>
       <c r="H68" s="11"/>
     </row>
@@ -3317,6 +3318,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="dfmXe0NuhKB6Z2HjBEGMmAvi85ZZuT1gtLSuIqL5QeCSHyxonOFt3kh8qLHs6FKdlTM9KPqtV/pE/mgZGwgDSw==" saltValue="zfIbWmM7LD6iB6BsXAZMHQ==" spinCount="100000" sheet="1" formatColumns="0" formatRows="0" insertRows="0"/>
   <mergeCells count="28">
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C53:H53"/>
+    <mergeCell ref="C56:H56"/>
+    <mergeCell ref="C60:H60"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="C2:E4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
     <mergeCell ref="E9:H9"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="E7:H7"/>
@@ -3331,20 +3346,6 @@
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="G15:G16"/>
     <mergeCell ref="H15:H16"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="C2:E4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="C53:H53"/>
-    <mergeCell ref="C56:H56"/>
-    <mergeCell ref="C60:H60"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -3407,19 +3408,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="900f5ea3-4309-4848-96c1-ad4c68ce6813">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06146d02-393f-48de-94b9-ef7e514a30fa" xsi:nil="true"/>
-    <_dlc_DocId xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">ETSV6M6J7ZTN-240384884-35593</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">
-      <Url>https://senaimt.sharepoint.com/sites/sfiemt/_layouts/15/DocIdRedir.aspx?ID=ETSV6M6J7ZTN-240384884-35593</Url>
-      <Description>ETSV6M6J7ZTN-240384884-35593</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3709,12 +3703,19 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="900f5ea3-4309-4848-96c1-ad4c68ce6813">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06146d02-393f-48de-94b9-ef7e514a30fa" xsi:nil="true"/>
+    <_dlc_DocId xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">ETSV6M6J7ZTN-240384884-35593</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">
+      <Url>https://senaimt.sharepoint.com/sites/sfiemt/_layouts/15/DocIdRedir.aspx?ID=ETSV6M6J7ZTN-240384884-35593</Url>
+      <Description>ETSV6M6J7ZTN-240384884-35593</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3726,12 +3727,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA13BBC6-8A75-4AE6-9EEA-9BB889D14091}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A6ECAD-A0AB-448D-840C-F95861E92F39}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="900f5ea3-4309-4848-96c1-ad4c68ce6813"/>
-    <ds:schemaRef ds:uri="06146d02-393f-48de-94b9-ef7e514a30fa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3756,9 +3754,12 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A6ECAD-A0AB-448D-840C-F95861E92F39}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA13BBC6-8A75-4AE6-9EEA-9BB889D14091}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="900f5ea3-4309-4848-96c1-ad4c68ce6813"/>
+    <ds:schemaRef ds:uri="06146d02-393f-48de-94b9-ef7e514a30fa"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>